<commit_message>
Textes J4 validés depuis la page contrôle
</commit_message>
<xml_diff>
--- a/textes_journee.xlsx
+++ b/textes_journee.xlsx
@@ -504,7 +504,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>match:J4:ACASA</t>
+          <t>une:J4</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -512,22 +512,22 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Essentiel du match</t>
+          <t>Titre de La Une</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>ACASA 4-3 Garges</t>
+          <t>Laval 5-4 Toulon</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>ACASA arrache la victoire face à Garges (4-3) sur un but de KIRTYS à la 39e, avec un doublé de Dianka.</t>
+          <t>9 buts entre Laval et Toulon</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>ACASA arrache la victoire face à Garges (4-3) sur un but de KIRTYS à la 39e, avec un doublé de DIANKA.</t>
+          <t>9 buts dans le choc entre Laval et Toulon</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
@@ -537,14 +537,14 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>but décisif à la 39e ; Bandyongou Dianka 2 buts</t>
+          <t>9 buts</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>match:J4:ARTISTES</t>
+          <t>match:J4:ACASA</t>
         </is>
       </c>
       <c r="B3" s="2" t="n">
@@ -557,17 +557,17 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Artistes 1-2 Nantes</t>
+          <t>ACASA 4-3 Garges</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>Nantes bat les Artistes 2-1.</t>
+          <t>ACASA arrache la victoire face à Garges (4-3) sur un but de KIRTYS à la 39e, avec un doublé de Dianka.</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>Nantes assure les 3 points contre les Artistes 2-1.</t>
+          <t>ACASA arrache la victoire face à Garges (4-3) sur un but de KIRTYS à la 39e, avec un doublé de DIANKA.</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
@@ -577,14 +577,14 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>victoire</t>
+          <t>but décisif à la 39e ; Bandyongou Dianka 2 buts</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>une:J4</t>
+          <t>match:J4:ARTISTES</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -592,22 +592,22 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Titre de La Une</t>
+          <t>Essentiel du match</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Laval 5-4 Toulon</t>
+          <t>Artistes 1-2 Nantes</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>9 buts entre Laval et Toulon</t>
+          <t>Nantes bat les Artistes 2-1.</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>9 buts dans le choc entre Laval et Toulon</t>
+          <t>Nantes assure les 3 points contre les Artistes 2-1.</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
@@ -617,7 +617,7 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>9 buts</t>
+          <t>victoire</t>
         </is>
       </c>
     </row>
@@ -767,10 +767,14 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>Toulouse arrache la victoire face au Sporting (3-2) sur un but d’ERRADAF à la 37e, avec deux passes décisives d’AZZAKHININI.</t>
-        </is>
-      </c>
-      <c r="G8" s="3" t="inlineStr"/>
+          <t>Toulouse arrache la victoire face au Sporting (3-2) sur un but d’ERRADDAF à la 37e, avec deux passes décisives d’AZZAKHNINI.</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
           <t>but décisif à la 37e ; Hamza Azzakhnini 2 passes</t>

</xml_diff>

<commit_message>
Textes J5 validés depuis la page contrôle
</commit_message>
<xml_diff>
--- a/textes_journee.xlsx
+++ b/textes_journee.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -504,11 +504,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>une:J4</t>
+          <t>une:J5</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
@@ -517,17 +517,17 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>Laval 5-4 Toulon</t>
+          <t>SPORTING 8-2 MONTPELLIER</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>9 buts entre Laval et Toulon</t>
+          <t>Dos Santos signe un quadruplé</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>9 buts dans le choc entre Laval et Toulon</t>
+          <t>Caio Dos Santos en feu signe un quadruplé et contribue au large succès du SPORTING</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
@@ -537,18 +537,18 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>9 buts</t>
+          <t>Caio Dos Santos 4 buts</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>match:J4:ACASA</t>
+          <t>match:J5:AVION</t>
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
@@ -557,17 +557,17 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>ACASA 4-3 Garges</t>
+          <t>AVION 2-3 LAVAL</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>ACASA arrache la victoire face à Garges (4-3) sur un but de KIRTYS à la 39e, avec un doublé de Dianka.</t>
+          <t>LAVAL bat AVION 3-2.</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>ACASA arrache la victoire face à Garges (4-3) sur un but de KIRTYS à la 39e, avec un doublé de DIANKA.</t>
+          <t>LAVAL se fait peur mais bat AVION 3-2.</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
@@ -577,18 +577,18 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>but décisif à la 39e ; Bandyongou Dianka 2 buts</t>
+          <t>victoire</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>match:J4:ARTISTES</t>
+          <t>match:J5:GARGES</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
@@ -597,17 +597,17 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Artistes 1-2 Nantes</t>
+          <t>GARGES 1-4 NICE</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Nantes bat les Artistes 2-1.</t>
+          <t>NICE bat GARGES 4-1, avec un doublé de De Araujo.</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>Nantes assure les 3 points contre les Artistes 2-1.</t>
+          <t>NICE bat GARGES 4-1, avec un doublé de De Araujo.</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
@@ -617,18 +617,18 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>victoire</t>
+          <t>victoire ; Fineo De Araujo 2 buts</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>match:J4:LAVAL</t>
+          <t>match:J5:GOAL</t>
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
@@ -637,17 +637,17 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Laval 5-4 Toulon</t>
+          <t>GOAL 5-3 TOULOUSE</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>Laval bat Toulon 5-4, avec un doublé de Guirio.</t>
+          <t>GOAL bat TOULOUSE 5-3, avec un doublé de Menendez.</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>Laval bat Toulon 5-4, avec un doublé de GUIRIO.</t>
+          <t>GOAL bat TOULOUSE 5-3, avec un doublé de Menendez et 2 cartons rouges côté lyonnais</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -657,18 +657,18 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>victoire ; Ouassini Guirio 2 buts</t>
+          <t>victoire ; Nicolas Menendez 2 buts</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>match:J4:MTP</t>
+          <t>match:J5:NANTES</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -677,17 +677,17 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Montpellier 4-4 Avion</t>
+          <t>NANTES 5-0 ACASA</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>Montpellier et Avion se quittent sur un nul 4-4, avec un triplé de Mesquita Rodrigues.</t>
+          <t>NANTES écarte ACASA 5-0 sans encaisser, avec deux passes décisives de Bendali.</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>Montpellier et Avion se quittent sur un nul 4-4, avec un triplé de MESQUITA.</t>
+          <t>NANTES ne laisse aucune chance à ACASA (5-0)</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
@@ -697,18 +697,18 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>nul ; David Mesquita Rodrigues 3 buts</t>
+          <t>victoire sans but encaissé ; Steve Bendali 2 passes</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>match:J4:NICE</t>
+          <t>match:J5:SPORTING</t>
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
@@ -717,17 +717,17 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Nice 2-5 Goal FC</t>
+          <t>SPORTING 8-2 MONTPELLIER</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>Goal FC bat Nice 5-2.</t>
+          <t>Large succès du Sporting contre MONTPELLIER (8-2), avec un quadruplé de Dos Santos.</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>Goal FC tient son rang face à Nice (5-2).</t>
+          <t>Large succès du Sporting contre MONTPELLIER (8-2), avec un quadruplé de Caio Dos Santos.</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
@@ -737,45 +737,325 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>victoire</t>
+          <t>écart de 6 ; Caio Dos Santos 4 buts</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
+          <t>match:J5:TOULON</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Essentiel du match</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>TOULON 3-3 ARTISTES</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>TOULON et les Artistes se quittent sur un nul 3-3, avec un doublé de Koita.</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>TOULON et les ARTISTES se quittent sur un nul 3-3, avec un doublé de Koita.</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>nul ; Ibrahim Koita 2 buts</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>une:J4</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Titre de La Une</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Laval 5-4 Toulon</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>9 buts entre Laval et Toulon</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>9 buts dans le choc entre Laval et Toulon</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>9 buts</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>match:J4:ACASA</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Essentiel du match</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>ACASA 4-3 Garges</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>ACASA arrache la victoire face à Garges (4-3) sur un but de KIRTYS à la 39e, avec un doublé de Dianka.</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>ACASA arrache la victoire face à Garges (4-3) sur un but de KIRTYS à la 39e, avec un doublé de DIANKA.</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>but décisif à la 39e ; Bandyongou Dianka 2 buts</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>match:J4:ARTISTES</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Essentiel du match</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Artistes 1-2 Nantes</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Nantes bat les Artistes 2-1.</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>Nantes assure les 3 points contre les Artistes 2-1.</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>victoire</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>match:J4:LAVAL</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Essentiel du match</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>Laval 5-4 Toulon</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>Laval bat Toulon 5-4, avec un doublé de Guirio.</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>Laval bat Toulon 5-4, avec un doublé de GUIRIO.</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>victoire ; Ouassini Guirio 2 buts</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>match:J4:MTP</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Essentiel du match</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Montpellier 4-4 Avion</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Montpellier et Avion se quittent sur un nul 4-4, avec un triplé de Mesquita Rodrigues.</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>Montpellier et Avion se quittent sur un nul 4-4, avec un triplé de MESQUITA.</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>nul ; David Mesquita Rodrigues 3 buts</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>match:J4:NICE</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Essentiel du match</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>Nice 2-5 Goal FC</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>Goal FC bat Nice 5-2.</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>Goal FC tient son rang face à Nice (5-2).</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>victoire</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
           <t>match:J4:TOULOUSE</t>
         </is>
       </c>
-      <c r="B8" s="2" t="n">
+      <c r="B15" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Essentiel du match</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Essentiel du match</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
         <is>
           <t>Toulouse 3-2 Sporting</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="E15" s="3" t="inlineStr">
         <is>
           <t>Toulouse arrache la victoire face au Sporting (3-2) sur un but d’Erraddaf à la 37e, avec deux passes décisives d’Azzakhnini.</t>
         </is>
       </c>
-      <c r="F8" s="4" t="inlineStr">
+      <c r="F15" s="4" t="inlineStr">
         <is>
           <t>Toulouse arrache la victoire face au Sporting (3-2) sur un but d’ERRADDAF à la 37e, avec deux passes décisives d’AZZAKHNINI.</t>
         </is>
       </c>
-      <c r="G8" s="3" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
         <is>
           <t>but décisif à la 37e ; Hamza Azzakhnini 2 passes</t>
         </is>
@@ -783,7 +1063,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="G2:G58" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G2:G65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"OK,A REVOIR"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Textes J1 validés depuis la page contrôle
</commit_message>
<xml_diff>
--- a/textes_journee.xlsx
+++ b/textes_journee.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:H22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1061,9 +1061,289 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>une:J1</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Titre de La Une</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>GOAL 5-4 NANTES</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>GOAL fait la différence en attaque placée</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>GOAL s’impose 5-4 contre NANTES mais a tremblé après avoir mené de quatre buts</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>4/5 attaque placée</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>match:J1:ACASA</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Essentiel du match</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>ACASA 5-0 AVION</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>ACASA écarte AVION 5-0 sans encaisser.</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>ACASA écrase AVION 5-0</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>victoire sans but encaissé</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>match:J1:GOAL</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Essentiel du match</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>GOAL 5-4 NANTES</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>GOAL s’impose 5-4 contre NANTES mais a tremblé après avoir mené de quatre buts, avec un doublé de Riano Garcia.</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>GOAL s'est fait peur mais prend les 3 pts à domicile</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>avance de 4 réduite à 1 ; Eduardo Riano Garcia 2 buts</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>match:J1:LAVAL</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Essentiel du match</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>LAVAL 7-2 NICE</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>Large succès de LAVAL contre NICE (7-2), avec un doublé de Bakkali.</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>Large succès de LAVAL contre NICE (7-2), avec un doublé de Bakkali.</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>écart de 5 ; Bilal Bakkali 2 buts</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>match:J1:SPORTING</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Essentiel du match</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>SPORTING 6-1 ARTISTES</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>Large succès du Sporting contre les Artistes (6-1), avec un quadruplé de Martinez Villalba.</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>Large succès du Sporting contre les Artistes (6-1), avec un quadruplé de Martinez Villalba.</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>écart de 5 ; Francisco Martinez Villalba 4 buts</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>match:J1:TOULON</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Essentiel du match</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>TOULON 5-3 GARGES</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>TOULON bat GARGES 5-3, avec un doublé de Dubois.</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>TOULON bat GARGES 5-3, avec un doublé de Dubois.</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>victoire ; Alexis Dubois 2 buts</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>match:J1:TOULOUSE</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Essentiel du match</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>TOULOUSE 3-4 MONTPELLIER</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>MONTPELLIER bat TOULOUSE 4-3, avec un doublé de Bouita.</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>MONTPELLIER bat TOULOUSE au terme d'un match très disputé</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>victoire ; Ayoub Bouita 2 buts</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="G2:G65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G2:G72" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"OK,A REVOIR"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Textes J2 validés depuis la page contrôle
</commit_message>
<xml_diff>
--- a/textes_journee.xlsx
+++ b/textes_journee.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:H29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1064,11 +1064,11 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>une:J1</t>
+          <t>une:J2</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
@@ -1077,17 +1077,17 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>GOAL 5-4 NANTES</t>
+          <t>TOULOUSE 3-5 LAVAL</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>GOAL fait la différence en attaque placée</t>
+          <t>LAVAL fait la différence en attaque placée</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>GOAL s’impose 5-4 contre NANTES mais a tremblé après avoir mené de quatre buts</t>
+          <t>LAVAL fait la différence en première mi-temps et sort victorieux contre TOULOUSE</t>
         </is>
       </c>
       <c r="G16" s="3" t="inlineStr">
@@ -1104,11 +1104,11 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>match:J1:ACASA</t>
+          <t>match:J2:ARTISTES</t>
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
@@ -1117,17 +1117,17 @@
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>ACASA 5-0 AVION</t>
+          <t>ARTISTES 3-4 GOAL</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>ACASA écarte AVION 5-0 sans encaisser.</t>
+          <t>Mené de deux buts, GOAL renverse les Artistes (4-3).</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>ACASA écrase AVION 5-0</t>
+          <t>Mené de deux buts, GOAL renverse les Artistes (4-3).</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
@@ -1137,18 +1137,18 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>victoire sans but encaissé</t>
+          <t>renversement après 2 buts de retard</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>match:J1:GOAL</t>
+          <t>match:J2:MTP</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
@@ -1157,17 +1157,17 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>GOAL 5-4 NANTES</t>
+          <t>MONTPELLIER 1-2 TOULON</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>GOAL s’impose 5-4 contre NANTES mais a tremblé après avoir mené de quatre buts, avec un doublé de Riano Garcia.</t>
+          <t>TOULON arrache la victoire face à MONTPELLIER (2-1) sur un but de Dubois à la 35e, avec deux passes décisives d’Ordonez Martin.</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>GOAL s'est fait peur mais prend les 3 pts à domicile</t>
+          <t>TOULON arrache la victoire face à MONTPELLIER (2-1) sur un but de Dubois à la 35e, avec deux passes décisives d’Ordonez Martin.</t>
         </is>
       </c>
       <c r="G18" s="3" t="inlineStr">
@@ -1177,18 +1177,18 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>avance de 4 réduite à 1 ; Eduardo Riano Garcia 2 buts</t>
+          <t>but décisif à la 35e ; Ruben Ordonez Martin 2 passes</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>match:J1:LAVAL</t>
+          <t>match:J2:NANTES</t>
         </is>
       </c>
       <c r="B19" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
@@ -1197,38 +1197,34 @@
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>LAVAL 7-2 NICE</t>
+          <t>NANTES 3-0 GARGES</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>Large succès de LAVAL contre NICE (7-2), avec un doublé de Bakkali.</t>
+          <t>NANTES bat GARGES 3-0 sans encaisser.</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>Large succès de LAVAL contre NICE (7-2), avec un doublé de Bakkali.</t>
-        </is>
-      </c>
-      <c r="G19" s="3" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
+          <t>NANTES bat GARGES 3-0 sans trembler</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr"/>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>écart de 5 ; Bilal Bakkali 2 buts</t>
+          <t>victoire sans but encaissé</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>match:J1:SPORTING</t>
+          <t>match:J2:NICE</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
@@ -1237,17 +1233,17 @@
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>SPORTING 6-1 ARTISTES</t>
+          <t>NICE 1-3 AVION</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>Large succès du Sporting contre les Artistes (6-1), avec un quadruplé de Martinez Villalba.</t>
+          <t>AVION bat NICE 3-1.</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>Large succès du Sporting contre les Artistes (6-1), avec un quadruplé de Martinez Villalba.</t>
+          <t>AVION tient sa première victoire de la saison face à NICE 3-1</t>
         </is>
       </c>
       <c r="G20" s="3" t="inlineStr">
@@ -1257,18 +1253,18 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>écart de 5 ; Francisco Martinez Villalba 4 buts</t>
+          <t>victoire</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>match:J1:TOULON</t>
+          <t>match:J2:SPORTING</t>
         </is>
       </c>
       <c r="B21" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
@@ -1277,17 +1273,17 @@
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>TOULON 5-3 GARGES</t>
+          <t>SPORTING 2-2 ACASA</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>TOULON bat GARGES 5-3, avec un doublé de Dubois.</t>
+          <t>Le Sporting et ACASA se quittent sur un nul 2-2.</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>TOULON bat GARGES 5-3, avec un doublé de Dubois.</t>
+          <t>Le SPORTING et ACASA se quittent sur un match nul 2-2.</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
@@ -1297,45 +1293,325 @@
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>victoire ; Alexis Dubois 2 buts</t>
+          <t>nul</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
+          <t>match:J2:TOULOUSE</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Essentiel du match</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>TOULOUSE 3-5 LAVAL</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>LAVAL s’impose 5-3 contre TOULOUSE mais a tremblé après avoir mené de cinq buts, avec un doublé de Bakkali.</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>LAVAL s’impose mais a tremblé après avoir mené de cinq buts, avec un doublé de Bakkali.</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>avance de 5 réduite à 2 ; Bilal Bakkali 2 buts</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>une:J1</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Titre de La Une</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>GOAL 5-4 NANTES</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>GOAL fait la différence en attaque placée</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>GOAL s’impose 5-4 contre NANTES mais a tremblé après avoir mené de quatre buts</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>4/5 attaque placée</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>match:J1:ACASA</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Essentiel du match</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>ACASA 5-0 AVION</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>ACASA écarte AVION 5-0 sans encaisser.</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>ACASA écrase AVION 5-0</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>victoire sans but encaissé</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>match:J1:GOAL</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Essentiel du match</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>GOAL 5-4 NANTES</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>GOAL s’impose 5-4 contre NANTES mais a tremblé après avoir mené de quatre buts, avec un doublé de Riano Garcia.</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>GOAL s'est fait peur mais prend les 3 pts à domicile</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>avance de 4 réduite à 1 ; Eduardo Riano Garcia 2 buts</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>match:J1:LAVAL</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Essentiel du match</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>LAVAL 7-2 NICE</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>Large succès de LAVAL contre NICE (7-2), avec un doublé de Bakkali.</t>
+        </is>
+      </c>
+      <c r="F26" s="4" t="inlineStr">
+        <is>
+          <t>Large succès de LAVAL contre NICE (7-2), avec un doublé de Bakkali.</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>écart de 5 ; Bilal Bakkali 2 buts</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>match:J1:SPORTING</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Essentiel du match</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>SPORTING 6-1 ARTISTES</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>Large succès du Sporting contre les Artistes (6-1), avec un quadruplé de Martinez Villalba.</t>
+        </is>
+      </c>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t>Large succès du Sporting contre les Artistes (6-1), avec un quadruplé de Martinez Villalba.</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>écart de 5 ; Francisco Martinez Villalba 4 buts</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>match:J1:TOULON</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Essentiel du match</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>TOULON 5-3 GARGES</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>TOULON bat GARGES 5-3, avec un doublé de Dubois.</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="inlineStr">
+        <is>
+          <t>TOULON bat GARGES 5-3, avec un doublé de Dubois.</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>victoire ; Alexis Dubois 2 buts</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
           <t>match:J1:TOULOUSE</t>
         </is>
       </c>
-      <c r="B22" s="2" t="n">
+      <c r="B29" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>Essentiel du match</t>
-        </is>
-      </c>
-      <c r="D22" s="3" t="inlineStr">
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Essentiel du match</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
         <is>
           <t>TOULOUSE 3-4 MONTPELLIER</t>
         </is>
       </c>
-      <c r="E22" s="3" t="inlineStr">
+      <c r="E29" s="3" t="inlineStr">
         <is>
           <t>MONTPELLIER bat TOULOUSE 4-3, avec un doublé de Bouita.</t>
         </is>
       </c>
-      <c r="F22" s="4" t="inlineStr">
+      <c r="F29" s="4" t="inlineStr">
         <is>
           <t>MONTPELLIER bat TOULOUSE au terme d'un match très disputé</t>
         </is>
       </c>
-      <c r="G22" s="3" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="H22" s="2" t="inlineStr">
+      <c r="G29" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
         <is>
           <t>victoire ; Ayoub Bouita 2 buts</t>
         </is>
@@ -1343,7 +1619,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="G2:G72" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G2:G79" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"OK,A REVOIR"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Textes J3 validés depuis la page contrôle
</commit_message>
<xml_diff>
--- a/textes_journee.xlsx
+++ b/textes_journee.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H29"/>
+  <dimension ref="A1:H36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1064,11 +1064,11 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>une:J2</t>
+          <t>une:J3</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
@@ -1077,17 +1077,17 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>TOULOUSE 3-5 LAVAL</t>
+          <t>GARGES 5-8 ARTISTES</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>LAVAL fait la différence en attaque placée</t>
+          <t>13 buts entre GARGES et les Artistes, record de la saison</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>LAVAL fait la différence en première mi-temps et sort victorieux contre TOULOUSE</t>
+          <t>13 buts entre GARGES et les Artistes, record de la saison</t>
         </is>
       </c>
       <c r="G16" s="3" t="inlineStr">
@@ -1097,18 +1097,18 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>4/5 attaque placée</t>
+          <t>record 13 buts</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>match:J2:ARTISTES</t>
+          <t>match:J3:AVION</t>
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
@@ -1117,17 +1117,17 @@
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>ARTISTES 3-4 GOAL</t>
+          <t>AVION 1-5 TOULOUSE</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>Mené de deux buts, GOAL renverse les Artistes (4-3).</t>
+          <t>Large succès de TOULOUSE contre AVION (5-1), avec un doublé d’Erraddaf.</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>Mené de deux buts, GOAL renverse les Artistes (4-3).</t>
+          <t>Large succès de TOULOUSE contre AVION (5-1), avec un doublé d’Erraddaf.</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
@@ -1137,18 +1137,18 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>renversement après 2 buts de retard</t>
+          <t>écart de 4 ; Yanis Erraddaf 2 buts</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>match:J2:MTP</t>
+          <t>match:J3:GARGES</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
@@ -1157,17 +1157,17 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>MONTPELLIER 1-2 TOULON</t>
+          <t>GARGES 5-8 ARTISTES</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>TOULON arrache la victoire face à MONTPELLIER (2-1) sur un but de Dubois à la 35e, avec deux passes décisives d’Ordonez Martin.</t>
+          <t>Les Artistes battent GARGES 8-5, avec un doublé de Sako. Avec 13 buts, c’est le match le plus prolifique de la saison.</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>TOULON arrache la victoire face à MONTPELLIER (2-1) sur un but de Dubois à la 35e, avec deux passes décisives d’Ordonez Martin.</t>
+          <t>Les ARTISTES sortent vainqueur avec un doublé de Sako.</t>
         </is>
       </c>
       <c r="G18" s="3" t="inlineStr">
@@ -1177,18 +1177,18 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>but décisif à la 35e ; Ruben Ordonez Martin 2 passes</t>
+          <t>victoire ; Mamadou Sako 2 buts ; record 13 buts</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>match:J2:NANTES</t>
+          <t>match:J3:GOAL</t>
         </is>
       </c>
       <c r="B19" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
@@ -1197,34 +1197,38 @@
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>NANTES 3-0 GARGES</t>
+          <t>GOAL 5-4 ACASA</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>NANTES bat GARGES 3-0 sans encaisser.</t>
+          <t>GOAL s’impose 5-4 contre ACASA mais a tremblé après avoir mené de cinq buts, avec un doublé de Toure.</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>NANTES bat GARGES 3-0 sans trembler</t>
-        </is>
-      </c>
-      <c r="G19" s="3" t="inlineStr"/>
+          <t>GOAL s’impose 5-4 contre ACASA mais a tremblé après avoir mené de cinq buts</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>victoire sans but encaissé</t>
+          <t>avance de 5 réduite à 1 ; Mamadou Toure 2 buts</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>match:J2:NICE</t>
+          <t>match:J3:LAVAL</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
@@ -1233,17 +1237,17 @@
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>NICE 1-3 AVION</t>
+          <t>LAVAL 4-3 MONTPELLIER</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>AVION bat NICE 3-1.</t>
+          <t>LAVAL arrache la victoire face à MONTPELLIER (4-3) sur un but de Megrous à la 37e.</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>AVION tient sa première victoire de la saison face à NICE 3-1</t>
+          <t>LAVAL arrache la victoire face à MONTPELLIER (4-3) sur un but de Megrous à la 37e.</t>
         </is>
       </c>
       <c r="G20" s="3" t="inlineStr">
@@ -1253,18 +1257,18 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>victoire</t>
+          <t>but décisif à la 37e</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>match:J2:SPORTING</t>
+          <t>match:J3:SPORTING</t>
         </is>
       </c>
       <c r="B21" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
@@ -1273,17 +1277,17 @@
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>SPORTING 2-2 ACASA</t>
+          <t>SPORTING 8-0 NICE</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>Le Sporting et ACASA se quittent sur un nul 2-2.</t>
+          <t>Le Sporting écarte NICE 8-0 sans encaisser, avec un doublé d’Amarilla Ortiz.</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>Le SPORTING et ACASA se quittent sur un match nul 2-2.</t>
+          <t>Le SPORTING pulvérise NICE 8-0</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
@@ -1293,18 +1297,18 @@
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>nul</t>
+          <t>victoire sans but encaissé ; Aldo Amarilla Ortiz 2 buts</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>match:J2:TOULOUSE</t>
+          <t>match:J3:TOULON</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
@@ -1313,17 +1317,17 @@
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>TOULOUSE 3-5 LAVAL</t>
+          <t>TOULON 7-3 NANTES</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>LAVAL s’impose 5-3 contre TOULOUSE mais a tremblé après avoir mené de cinq buts, avec un doublé de Bakkali.</t>
+          <t>Large succès de TOULON contre NANTES (7-3), avec un triplé de Dubois.</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>LAVAL s’impose mais a tremblé après avoir mené de cinq buts, avec un doublé de Bakkali.</t>
+          <t>Large succès de TOULON contre NANTES (7-3), avec un triplé de Dubois.</t>
         </is>
       </c>
       <c r="G22" s="3" t="inlineStr">
@@ -1333,18 +1337,18 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>avance de 5 réduite à 2 ; Bilal Bakkali 2 buts</t>
+          <t>écart de 4 ; Alexis Dubois 3 buts</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>une:J1</t>
+          <t>une:J2</t>
         </is>
       </c>
       <c r="B23" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
@@ -1353,17 +1357,17 @@
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>GOAL 5-4 NANTES</t>
+          <t>TOULOUSE 3-5 LAVAL</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>GOAL fait la différence en attaque placée</t>
+          <t>LAVAL fait la différence en attaque placée</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>GOAL s’impose 5-4 contre NANTES mais a tremblé après avoir mené de quatre buts</t>
+          <t>LAVAL fait la différence en première mi-temps et sort victorieux contre TOULOUSE</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
@@ -1380,11 +1384,11 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>match:J1:ACASA</t>
+          <t>match:J2:ARTISTES</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
@@ -1393,17 +1397,17 @@
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>ACASA 5-0 AVION</t>
+          <t>ARTISTES 3-4 GOAL</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>ACASA écarte AVION 5-0 sans encaisser.</t>
+          <t>Mené de deux buts, GOAL renverse les Artistes (4-3).</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>ACASA écrase AVION 5-0</t>
+          <t>Mené de deux buts, GOAL renverse les Artistes (4-3).</t>
         </is>
       </c>
       <c r="G24" s="3" t="inlineStr">
@@ -1413,18 +1417,18 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>victoire sans but encaissé</t>
+          <t>renversement après 2 buts de retard</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>match:J1:GOAL</t>
+          <t>match:J2:MTP</t>
         </is>
       </c>
       <c r="B25" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
@@ -1433,17 +1437,17 @@
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>GOAL 5-4 NANTES</t>
+          <t>MONTPELLIER 1-2 TOULON</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>GOAL s’impose 5-4 contre NANTES mais a tremblé après avoir mené de quatre buts, avec un doublé de Riano Garcia.</t>
+          <t>TOULON arrache la victoire face à MONTPELLIER (2-1) sur un but de Dubois à la 35e, avec deux passes décisives d’Ordonez Martin.</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>GOAL s'est fait peur mais prend les 3 pts à domicile</t>
+          <t>TOULON arrache la victoire face à MONTPELLIER (2-1) sur un but de Dubois à la 35e, avec deux passes décisives d’Ordonez Martin.</t>
         </is>
       </c>
       <c r="G25" s="3" t="inlineStr">
@@ -1453,18 +1457,18 @@
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>avance de 4 réduite à 1 ; Eduardo Riano Garcia 2 buts</t>
+          <t>but décisif à la 35e ; Ruben Ordonez Martin 2 passes</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>match:J1:LAVAL</t>
+          <t>match:J2:NANTES</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
@@ -1473,38 +1477,34 @@
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>LAVAL 7-2 NICE</t>
+          <t>NANTES 3-0 GARGES</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>Large succès de LAVAL contre NICE (7-2), avec un doublé de Bakkali.</t>
+          <t>NANTES bat GARGES 3-0 sans encaisser.</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>Large succès de LAVAL contre NICE (7-2), avec un doublé de Bakkali.</t>
-        </is>
-      </c>
-      <c r="G26" s="3" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
+          <t>NANTES bat GARGES 3-0 sans trembler</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr"/>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>écart de 5 ; Bilal Bakkali 2 buts</t>
+          <t>victoire sans but encaissé</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>match:J1:SPORTING</t>
+          <t>match:J2:NICE</t>
         </is>
       </c>
       <c r="B27" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
@@ -1513,17 +1513,17 @@
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>SPORTING 6-1 ARTISTES</t>
+          <t>NICE 1-3 AVION</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>Large succès du Sporting contre les Artistes (6-1), avec un quadruplé de Martinez Villalba.</t>
+          <t>AVION bat NICE 3-1.</t>
         </is>
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>Large succès du Sporting contre les Artistes (6-1), avec un quadruplé de Martinez Villalba.</t>
+          <t>AVION tient sa première victoire de la saison face à NICE 3-1</t>
         </is>
       </c>
       <c r="G27" s="3" t="inlineStr">
@@ -1533,18 +1533,18 @@
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>écart de 5 ; Francisco Martinez Villalba 4 buts</t>
+          <t>victoire</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>match:J1:TOULON</t>
+          <t>match:J2:SPORTING</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
@@ -1553,17 +1553,17 @@
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>TOULON 5-3 GARGES</t>
+          <t>SPORTING 2-2 ACASA</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>TOULON bat GARGES 5-3, avec un doublé de Dubois.</t>
+          <t>Le Sporting et ACASA se quittent sur un nul 2-2.</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>TOULON bat GARGES 5-3, avec un doublé de Dubois.</t>
+          <t>Le SPORTING et ACASA se quittent sur un match nul 2-2.</t>
         </is>
       </c>
       <c r="G28" s="3" t="inlineStr">
@@ -1573,45 +1573,325 @@
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>victoire ; Alexis Dubois 2 buts</t>
+          <t>nul</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
+          <t>match:J2:TOULOUSE</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Essentiel du match</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>TOULOUSE 3-5 LAVAL</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>LAVAL s’impose 5-3 contre TOULOUSE mais a tremblé après avoir mené de cinq buts, avec un doublé de Bakkali.</t>
+        </is>
+      </c>
+      <c r="F29" s="4" t="inlineStr">
+        <is>
+          <t>LAVAL s’impose mais a tremblé après avoir mené de cinq buts, avec un doublé de Bakkali.</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>avance de 5 réduite à 2 ; Bilal Bakkali 2 buts</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>une:J1</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Titre de La Une</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>GOAL 5-4 NANTES</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>GOAL fait la différence en attaque placée</t>
+        </is>
+      </c>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>GOAL s’impose 5-4 contre NANTES mais a tremblé après avoir mené de quatre buts</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>4/5 attaque placée</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>match:J1:ACASA</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Essentiel du match</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>ACASA 5-0 AVION</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>ACASA écarte AVION 5-0 sans encaisser.</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="inlineStr">
+        <is>
+          <t>ACASA écrase AVION 5-0</t>
+        </is>
+      </c>
+      <c r="G31" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>victoire sans but encaissé</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>match:J1:GOAL</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Essentiel du match</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>GOAL 5-4 NANTES</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>GOAL s’impose 5-4 contre NANTES mais a tremblé après avoir mené de quatre buts, avec un doublé de Riano Garcia.</t>
+        </is>
+      </c>
+      <c r="F32" s="4" t="inlineStr">
+        <is>
+          <t>GOAL s'est fait peur mais prend les 3 pts à domicile</t>
+        </is>
+      </c>
+      <c r="G32" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>avance de 4 réduite à 1 ; Eduardo Riano Garcia 2 buts</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>match:J1:LAVAL</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>Essentiel du match</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>LAVAL 7-2 NICE</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>Large succès de LAVAL contre NICE (7-2), avec un doublé de Bakkali.</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>Large succès de LAVAL contre NICE (7-2), avec un doublé de Bakkali.</t>
+        </is>
+      </c>
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>écart de 5 ; Bilal Bakkali 2 buts</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>match:J1:SPORTING</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Essentiel du match</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>SPORTING 6-1 ARTISTES</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>Large succès du Sporting contre les Artistes (6-1), avec un quadruplé de Martinez Villalba.</t>
+        </is>
+      </c>
+      <c r="F34" s="4" t="inlineStr">
+        <is>
+          <t>Large succès du Sporting contre les Artistes (6-1), avec un quadruplé de Martinez Villalba.</t>
+        </is>
+      </c>
+      <c r="G34" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>écart de 5 ; Francisco Martinez Villalba 4 buts</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>match:J1:TOULON</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>Essentiel du match</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>TOULON 5-3 GARGES</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>TOULON bat GARGES 5-3, avec un doublé de Dubois.</t>
+        </is>
+      </c>
+      <c r="F35" s="4" t="inlineStr">
+        <is>
+          <t>TOULON bat GARGES 5-3, avec un doublé de Dubois.</t>
+        </is>
+      </c>
+      <c r="G35" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>victoire ; Alexis Dubois 2 buts</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
           <t>match:J1:TOULOUSE</t>
         </is>
       </c>
-      <c r="B29" s="2" t="n">
+      <c r="B36" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="C29" s="2" t="inlineStr">
-        <is>
-          <t>Essentiel du match</t>
-        </is>
-      </c>
-      <c r="D29" s="3" t="inlineStr">
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Essentiel du match</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
         <is>
           <t>TOULOUSE 3-4 MONTPELLIER</t>
         </is>
       </c>
-      <c r="E29" s="3" t="inlineStr">
+      <c r="E36" s="3" t="inlineStr">
         <is>
           <t>MONTPELLIER bat TOULOUSE 4-3, avec un doublé de Bouita.</t>
         </is>
       </c>
-      <c r="F29" s="4" t="inlineStr">
+      <c r="F36" s="4" t="inlineStr">
         <is>
           <t>MONTPELLIER bat TOULOUSE au terme d'un match très disputé</t>
         </is>
       </c>
-      <c r="G29" s="3" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="H29" s="2" t="inlineStr">
+      <c r="G36" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
         <is>
           <t>victoire ; Ayoub Bouita 2 buts</t>
         </is>
@@ -1619,7 +1899,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="G2:G79" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G2:G86" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"OK,A REVOIR"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>